<commit_message>
feat: enhance notes handling in FocusViewWindow and ScanWindow to prevent saving placeholder text
</commit_message>
<xml_diff>
--- a/Sessions/test/3rd October session 1.xlsx
+++ b/Sessions/test/3rd October session 1.xlsx
@@ -767,11 +767,7 @@
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Add notes here...</t>
-        </is>
-      </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>excel_import</t>

</xml_diff>